<commit_message>
docs: update excel and diagram for v2.1
</commit_message>
<xml_diff>
--- a/Documents/Controlled_Vocabularies_Instructions.xlsx
+++ b/Documents/Controlled_Vocabularies_Instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29421"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri.sharepoint.com/sites/hri-team022/Shared Documents/05 - FAIR/Workplan &amp; Activities/2025/D1_Metadata, data modeling and library/1.Metadata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{027CF694-BCEA-4479-A1BF-AC0FDE82ED29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C2AB57-AA95-FC4A-A068-34078EB00E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C3D56D4C-58DE-344E-9B77-FB88BD7D2C37}"/>
+    <workbookView xWindow="6120" yWindow="-17240" windowWidth="26440" windowHeight="13700" xr2:uid="{C3D56D4C-58DE-344E-9B77-FB88BD7D2C37}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <author>tc={CDD8962E-205D-8B4E-9500-F90E76A24498}</author>
   </authors>
   <commentList>
-    <comment ref="G14" authorId="0" shapeId="0" xr:uid="{1B004A23-1A9A-3B44-851E-684A25CDFD43}">
+    <comment ref="G15" authorId="0" shapeId="0" xr:uid="{1B004A23-1A9A-3B44-851E-684A25CDFD43}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -50,7 +50,7 @@
     Is this still correct? According to HealthDCAT point to class License Document and add type from ADMS type vocabulary </t>
       </text>
     </comment>
-    <comment ref="D17" authorId="1" shapeId="0" xr:uid="{CDD8962E-205D-8B4E-9500-F90E76A24498}">
+    <comment ref="D18" authorId="1" shapeId="0" xr:uid="{CDD8962E-205D-8B4E-9500-F90E76A24498}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="201">
   <si>
     <t>Class</t>
   </si>
@@ -770,12 +770,66 @@
     spdx:algorithm spdx:checksumAlgorithm_md5 ;
     spdx:checksumValue "5d41402abc4b2a76b9719d911017c592"^^xsd:hexBinary .</t>
   </si>
+  <si>
+    <t>availability</t>
+  </si>
+  <si>
+    <t>dcatap:availability</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/planned-availability</t>
+  </si>
+  <si>
+    <t>Choose the availability of the Distribution from the EU Authority table.</t>
+  </si>
+  <si>
+    <t>http://publications.europa.eu/resource/authority/planned-availability/AVAILABLE</t>
+  </si>
+  <si>
+    <t>&lt;http://example.healthdata.nl/set/distribution&gt; dcatap:availability &lt;http://publications.europa.eu/resource/authority/planned-availability/AVAILABLE&gt;.</t>
+  </si>
+  <si>
+    <t>https://op.europa.eu/en/web/eu-vocabularies/dataset/-/resource?uri=http://publications.europa.eu/resource/dataset/planned-availability</t>
+  </si>
+  <si>
+    <t>anatomical location covered</t>
+  </si>
+  <si>
+    <t>hri:anatomicalLocationCovered</t>
+  </si>
+  <si>
+    <t>Children of http://snomed.info/id/91723000</t>
+  </si>
+  <si>
+    <t>Select the relevant anatomical structure from SNOMED CT. Multiple anatomical locations can be provided.</t>
+  </si>
+  <si>
+    <t>http://snomed.info/id/39607008</t>
+  </si>
+  <si>
+    <t>&lt;http://example.healthdata.nl/set/dataset&gt; hri:anatomicalLocationCovered                &lt;http://snomed.info/id/39607008&gt;.</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>https://hdeu-dcat.data.health.europa.eu/resource/authority/health-activity</t>
+  </si>
+  <si>
+    <t>https://hdeu-dcat.data.health.europa.eu/resource/authority/health-activity/HEALTH_REGISTRIES</t>
+  </si>
+  <si>
+    <t>&lt;http://example.healthdata.nl/set/activity&gt; dct:type &lt;https://hdeu-dcat.data.health.europa.eu/resource/authority/health-activity/HEALTH_REGISTRIES&gt;.</t>
+  </si>
+  <si>
+    <t>Choose the type of the activity from the Health Activity controlled vocabulary.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -866,7 +920,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -899,6 +953,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1048,8 +1103,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{476EE117-E9DA-6848-A569-D444A297C9B5}" name="Table1" displayName="Table1" ref="A1:H35" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H35" xr:uid="{476EE117-E9DA-6848-A569-D444A297C9B5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{476EE117-E9DA-6848-A569-D444A297C9B5}" name="Table1" displayName="Table1" ref="A1:H38" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H38" xr:uid="{476EE117-E9DA-6848-A569-D444A297C9B5}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{6C8BE34C-2226-BD4F-B7F5-34DC9F76FBB0}" name="Class" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{57591C71-E14B-BC47-B4DA-F5206AA15D23}" name="Property label" dataDxfId="6"/>
@@ -1381,10 +1436,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="G14" dT="2025-10-02T14:31:39.93" personId="{9C0D1E49-CD60-FC4E-BB42-D6566C1A8822}" id="{1B004A23-1A9A-3B44-851E-684A25CDFD43}">
+  <threadedComment ref="G15" dT="2025-10-02T14:31:39.93" personId="{9C0D1E49-CD60-FC4E-BB42-D6566C1A8822}" id="{1B004A23-1A9A-3B44-851E-684A25CDFD43}">
     <text xml:space="preserve">Is this still correct? According to HealthDCAT point to class License Document and add type from ADMS type vocabulary </text>
   </threadedComment>
-  <threadedComment ref="D17" dT="2025-10-02T14:57:02.53" personId="{9C0D1E49-CD60-FC4E-BB42-D6566C1A8822}" id="{CDD8962E-205D-8B4E-9500-F90E76A24498}">
+  <threadedComment ref="D18" dT="2025-10-02T14:57:02.53" personId="{9C0D1E49-CD60-FC4E-BB42-D6566C1A8822}" id="{CDD8962E-205D-8B4E-9500-F90E76A24498}">
     <text>New vocabulary published in release 5: http://13.81.34.152:1101/resource/authority/publisher-type</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -1398,20 +1453,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82062278-CD36-1E48-9DF1-1ABFED2CE0C5}">
-  <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="20.375" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="52.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="62.625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="67.375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="67.375" customWidth="1"/>
-    <col min="8" max="8" width="50.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="30.5" customWidth="1"/>
+    <col min="4" max="4" width="52.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="67.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="67.33203125" customWidth="1"/>
+    <col min="8" max="8" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="24">
+    <row r="1" spans="1:8" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1437,7 +1492,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="108.75">
+    <row r="2" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
@@ -1463,886 +1518,967 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="54.75">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="408" customHeight="1">
+      <c r="B3" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>27</v>
+        <v>17</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="46.5">
+        <v>21</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="408" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>34</v>
+        <v>24</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="163.5">
+        <v>28</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" ht="90.75">
+        <v>35</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" ht="72.75">
+    <row r="8" spans="1:8" ht="100" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" ht="54.75">
+    <row r="9" spans="1:8" ht="80" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="90.75">
+        <v>54</v>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="54.75">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="100" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H12" s="12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="199.5">
-      <c r="A12" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="46.5">
+    <row r="13" spans="1:8" ht="280" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>76</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>34</v>
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="90.75">
+        <v>79</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>76</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="100" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" ht="46.5">
-      <c r="A15" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="126.75">
+      <c r="H15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>97</v>
+        <v>24</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="1:8" ht="54.75">
+        <v>93</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="140" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>104</v>
+        <v>96</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>100</v>
       </c>
       <c r="H17" s="7"/>
     </row>
-    <row r="18" spans="1:8" ht="36">
+    <row r="18" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>103</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>105</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" ht="36">
-      <c r="A19" s="5" t="s">
+      <c r="H19" s="7"/>
+    </row>
+    <row r="20" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" ht="46.5">
-      <c r="A20" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>117</v>
+      <c r="B20" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>184</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>119</v>
+        <v>185</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>186</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>121</v>
+        <v>187</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="46.5">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>31</v>
+        <v>111</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>123</v>
+        <v>112</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>113</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="88.5" customHeight="1">
+        <v>114</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" ht="36">
+        <v>118</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>127</v>
+        <v>30</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>128</v>
+        <v>31</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>129</v>
+        <v>32</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" ht="54.75">
+        <v>34</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>132</v>
+        <v>82</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>136</v>
+        <v>84</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="H24" s="7"/>
     </row>
-    <row r="25" spans="1:8" ht="54.75">
+    <row r="25" spans="1:8" ht="40" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="H25" s="7"/>
+    </row>
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F27" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G27" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="H25" s="12" t="s">
+      <c r="H27" s="12" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="54.75">
-      <c r="A26" s="5" t="s">
+    <row r="28" spans="1:8" ht="80" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E28" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F28" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G28" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="H28" s="12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="199.5">
-      <c r="A27" s="5" t="s">
+    <row r="29" spans="1:8" ht="280" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B29" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C29" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F29" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H29" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="54.75">
-      <c r="A28" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="H28" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="46.5">
-      <c r="A29" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="H29" s="12" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="46.5">
+    <row r="30" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>150</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>157</v>
+        <v>11</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>151</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>153</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="90.75">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>150</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>159</v>
+        <v>118</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>154</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="H31" s="7"/>
-    </row>
-    <row r="32" spans="1:8" ht="46.5">
+        <v>155</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="69" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>150</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="100" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="H33" s="7"/>
+    </row>
+    <row r="34" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D34" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E34" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F34" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H32" s="12" t="s">
+      <c r="H34" s="12" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="90.75">
-      <c r="A33" s="5" t="s">
+    <row r="35" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B35" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D35" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E35" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F35" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="G35" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" ht="90.75">
-      <c r="A34" s="5" t="s">
+      <c r="H35" s="7"/>
+    </row>
+    <row r="36" spans="1:8" ht="140" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B36" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D36" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E36" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F36" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="G34" s="7" t="s">
+      <c r="G36" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:8" ht="72.75">
-      <c r="A35" s="5" t="s">
+      <c r="H36" s="7"/>
+    </row>
+    <row r="37" spans="1:8" ht="80" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B37" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D37" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E37" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F37" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="G37" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="H35" s="7"/>
+      <c r="H37" s="7"/>
+    </row>
+    <row r="38" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H38" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{F13AD9A4-4C4B-CB47-8643-96F5DC715F97}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{39E26470-555B-E44D-836C-FD734685EB62}"/>
-    <hyperlink ref="D5" r:id="rId3" xr:uid="{886DEB45-C5C7-D74C-82B2-F54D3ABCAE0C}"/>
-    <hyperlink ref="D6" r:id="rId4" location="vocab-legal-basis" xr:uid="{A0A1990B-215A-7C4B-BC66-D1B38C115F5F}"/>
-    <hyperlink ref="D7" r:id="rId5" xr:uid="{87D883FE-76CE-6F4F-BDC4-15519F0B8399}"/>
-    <hyperlink ref="D8" r:id="rId6" location="vocab-purposes" xr:uid="{6A57CF52-B7E4-FB4B-9DF0-83E7CC279B3B}"/>
-    <hyperlink ref="D9" r:id="rId7" xr:uid="{77563F54-99C2-C74F-BB0A-28F9F9B42F92}"/>
-    <hyperlink ref="D10" r:id="rId8" xr:uid="{15BA4E60-9F74-B043-B774-48EEACD44EAC}"/>
-    <hyperlink ref="D11" r:id="rId9" xr:uid="{DA5AE8B5-AE13-8343-AB34-85D4AC379459}"/>
-    <hyperlink ref="D14" r:id="rId10" xr:uid="{A50977BC-2BF2-C948-96BB-23BFB2C5D1AF}"/>
-    <hyperlink ref="D15" r:id="rId11" xr:uid="{F6844650-940E-8242-8D59-7AB95C861BAD}"/>
-    <hyperlink ref="D18" r:id="rId12" xr:uid="{9901F250-A9AF-164C-8EA7-F1628EF6F615}"/>
-    <hyperlink ref="D20" r:id="rId13" xr:uid="{9FEF903E-6DF7-A64A-970F-608BCBF3ED08}"/>
-    <hyperlink ref="D19" r:id="rId14" xr:uid="{1DE9ACCD-73FD-824F-A4B8-FC7C0A9297F9}"/>
-    <hyperlink ref="D23" r:id="rId15" xr:uid="{0C102235-C1FE-DF4E-9EF0-452A8C4B99F3}"/>
-    <hyperlink ref="D24" r:id="rId16" xr:uid="{6680C7E5-A8CD-704E-BB19-425DBE804DF1}"/>
-    <hyperlink ref="D25" r:id="rId17" xr:uid="{5B8D47C9-3364-CD4F-906B-B4A9C3351E33}"/>
-    <hyperlink ref="D26" r:id="rId18" xr:uid="{693A02CE-9CD2-FC4F-BEE4-7B3E8FC4C3F0}"/>
-    <hyperlink ref="D28" r:id="rId19" xr:uid="{04C3D598-6726-8C41-839F-4871DE0665E1}"/>
-    <hyperlink ref="D29" r:id="rId20" xr:uid="{185964F3-ED25-B944-B088-4B2F96AFA396}"/>
-    <hyperlink ref="D32" r:id="rId21" xr:uid="{F217914E-3C0F-3841-B206-EA5DB70AFB2B}"/>
-    <hyperlink ref="D33" r:id="rId22" location="table-1-credit-terms-and-urls" xr:uid="{E5EC8DE6-5CB5-F444-A584-18D46550321A}"/>
-    <hyperlink ref="D35" r:id="rId23" location="d4e2129" xr:uid="{CE5FD63E-3726-6341-94B9-3DF727F02999}"/>
-    <hyperlink ref="D13" r:id="rId24" xr:uid="{CC832F52-80C7-A94A-A421-910576DC4DDB}"/>
-    <hyperlink ref="D17" r:id="rId25" xr:uid="{B4CAB58E-0550-CD4E-937D-1423E83695F7}"/>
-    <hyperlink ref="D21" r:id="rId26" xr:uid="{D84949F3-B710-7E43-A43F-09C5C9C360DC}"/>
-    <hyperlink ref="D22" r:id="rId27" xr:uid="{44ACA96E-DD48-944D-840A-0283433ED864}"/>
-    <hyperlink ref="D30" r:id="rId28" xr:uid="{54D8F0D2-D841-3F47-9037-BE54E1AA8D59}"/>
-    <hyperlink ref="D31" r:id="rId29" xr:uid="{1D692552-EA84-FE40-B836-4C34136F4CDF}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{39E26470-555B-E44D-836C-FD734685EB62}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{886DEB45-C5C7-D74C-82B2-F54D3ABCAE0C}"/>
+    <hyperlink ref="D7" r:id="rId4" location="vocab-legal-basis" xr:uid="{A0A1990B-215A-7C4B-BC66-D1B38C115F5F}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{87D883FE-76CE-6F4F-BDC4-15519F0B8399}"/>
+    <hyperlink ref="D9" r:id="rId6" location="vocab-purposes" xr:uid="{6A57CF52-B7E4-FB4B-9DF0-83E7CC279B3B}"/>
+    <hyperlink ref="D10" r:id="rId7" xr:uid="{77563F54-99C2-C74F-BB0A-28F9F9B42F92}"/>
+    <hyperlink ref="D11" r:id="rId8" xr:uid="{15BA4E60-9F74-B043-B774-48EEACD44EAC}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{DA5AE8B5-AE13-8343-AB34-85D4AC379459}"/>
+    <hyperlink ref="D15" r:id="rId10" xr:uid="{A50977BC-2BF2-C948-96BB-23BFB2C5D1AF}"/>
+    <hyperlink ref="D16" r:id="rId11" xr:uid="{F6844650-940E-8242-8D59-7AB95C861BAD}"/>
+    <hyperlink ref="D19" r:id="rId12" xr:uid="{9901F250-A9AF-164C-8EA7-F1628EF6F615}"/>
+    <hyperlink ref="D22" r:id="rId13" xr:uid="{9FEF903E-6DF7-A64A-970F-608BCBF3ED08}"/>
+    <hyperlink ref="D21" r:id="rId14" xr:uid="{1DE9ACCD-73FD-824F-A4B8-FC7C0A9297F9}"/>
+    <hyperlink ref="D25" r:id="rId15" xr:uid="{0C102235-C1FE-DF4E-9EF0-452A8C4B99F3}"/>
+    <hyperlink ref="D26" r:id="rId16" xr:uid="{6680C7E5-A8CD-704E-BB19-425DBE804DF1}"/>
+    <hyperlink ref="D27" r:id="rId17" xr:uid="{5B8D47C9-3364-CD4F-906B-B4A9C3351E33}"/>
+    <hyperlink ref="D28" r:id="rId18" xr:uid="{693A02CE-9CD2-FC4F-BEE4-7B3E8FC4C3F0}"/>
+    <hyperlink ref="D30" r:id="rId19" xr:uid="{04C3D598-6726-8C41-839F-4871DE0665E1}"/>
+    <hyperlink ref="D31" r:id="rId20" xr:uid="{185964F3-ED25-B944-B088-4B2F96AFA396}"/>
+    <hyperlink ref="D34" r:id="rId21" xr:uid="{F217914E-3C0F-3841-B206-EA5DB70AFB2B}"/>
+    <hyperlink ref="D35" r:id="rId22" location="table-1-credit-terms-and-urls" xr:uid="{E5EC8DE6-5CB5-F444-A584-18D46550321A}"/>
+    <hyperlink ref="D37" r:id="rId23" location="d4e2129" xr:uid="{CE5FD63E-3726-6341-94B9-3DF727F02999}"/>
+    <hyperlink ref="D14" r:id="rId24" xr:uid="{CC832F52-80C7-A94A-A421-910576DC4DDB}"/>
+    <hyperlink ref="D18" r:id="rId25" xr:uid="{B4CAB58E-0550-CD4E-937D-1423E83695F7}"/>
+    <hyperlink ref="D23" r:id="rId26" xr:uid="{D84949F3-B710-7E43-A43F-09C5C9C360DC}"/>
+    <hyperlink ref="D24" r:id="rId27" xr:uid="{44ACA96E-DD48-944D-840A-0283433ED864}"/>
+    <hyperlink ref="D32" r:id="rId28" xr:uid="{54D8F0D2-D841-3F47-9037-BE54E1AA8D59}"/>
+    <hyperlink ref="D33" r:id="rId29" xr:uid="{1D692552-EA84-FE40-B836-4C34136F4CDF}"/>
     <hyperlink ref="H2" r:id="rId30" xr:uid="{2F0E098F-4E5A-43DF-AAFE-BC2C783D99E7}"/>
-    <hyperlink ref="H3" r:id="rId31" xr:uid="{28E65107-BF8D-4049-958F-FD53912FDA27}"/>
-    <hyperlink ref="H5" r:id="rId32" xr:uid="{24BE1DEF-D408-40EC-B029-0888D4BEF2CB}"/>
-    <hyperlink ref="H9" r:id="rId33" xr:uid="{0C983183-5591-4945-BDEF-74B7775B2B41}"/>
-    <hyperlink ref="H10" r:id="rId34" xr:uid="{45D23874-CCA6-421F-82B9-6E93BA1E0820}"/>
-    <hyperlink ref="H11" r:id="rId35" xr:uid="{EFE5F203-DF87-4D93-BF6C-4AF347FE8F90}"/>
-    <hyperlink ref="H13" r:id="rId36" xr:uid="{8BC37844-7C2F-416E-99AD-56A916D16991}"/>
-    <hyperlink ref="H15" r:id="rId37" xr:uid="{4437386F-9D50-4865-9E43-6A6597BEAA6B}"/>
-    <hyperlink ref="H20" r:id="rId38" xr:uid="{8F701DF3-57F6-46C5-A854-BF2ACDB3DBE8}"/>
-    <hyperlink ref="H21" r:id="rId39" xr:uid="{3CFE251B-5CCE-4977-B78B-81C849A93D63}"/>
-    <hyperlink ref="H25" r:id="rId40" xr:uid="{1DE24D30-7878-43F9-949A-B154C1684233}"/>
-    <hyperlink ref="H26" r:id="rId41" xr:uid="{9B59E434-E624-4038-B753-DC5BD9DF8609}"/>
-    <hyperlink ref="H28" r:id="rId42" xr:uid="{57E3D166-5B64-4BF1-A7D3-39C0EC43DCC8}"/>
-    <hyperlink ref="H29" r:id="rId43" xr:uid="{1AA839FE-7FAE-4414-89EC-EE37E17E27B6}"/>
-    <hyperlink ref="H30" r:id="rId44" xr:uid="{8920AF35-BAAB-4C2A-B1BC-98F0255C4797}"/>
-    <hyperlink ref="H32" r:id="rId45" xr:uid="{C4D06269-938A-498A-88B2-93547914AA0E}"/>
+    <hyperlink ref="H4" r:id="rId31" xr:uid="{28E65107-BF8D-4049-958F-FD53912FDA27}"/>
+    <hyperlink ref="H6" r:id="rId32" xr:uid="{24BE1DEF-D408-40EC-B029-0888D4BEF2CB}"/>
+    <hyperlink ref="H10" r:id="rId33" xr:uid="{0C983183-5591-4945-BDEF-74B7775B2B41}"/>
+    <hyperlink ref="H11" r:id="rId34" xr:uid="{45D23874-CCA6-421F-82B9-6E93BA1E0820}"/>
+    <hyperlink ref="H12" r:id="rId35" xr:uid="{EFE5F203-DF87-4D93-BF6C-4AF347FE8F90}"/>
+    <hyperlink ref="H14" r:id="rId36" xr:uid="{8BC37844-7C2F-416E-99AD-56A916D16991}"/>
+    <hyperlink ref="H16" r:id="rId37" xr:uid="{4437386F-9D50-4865-9E43-6A6597BEAA6B}"/>
+    <hyperlink ref="H22" r:id="rId38" xr:uid="{8F701DF3-57F6-46C5-A854-BF2ACDB3DBE8}"/>
+    <hyperlink ref="H23" r:id="rId39" xr:uid="{3CFE251B-5CCE-4977-B78B-81C849A93D63}"/>
+    <hyperlink ref="H27" r:id="rId40" xr:uid="{1DE24D30-7878-43F9-949A-B154C1684233}"/>
+    <hyperlink ref="H28" r:id="rId41" xr:uid="{9B59E434-E624-4038-B753-DC5BD9DF8609}"/>
+    <hyperlink ref="H30" r:id="rId42" xr:uid="{57E3D166-5B64-4BF1-A7D3-39C0EC43DCC8}"/>
+    <hyperlink ref="H31" r:id="rId43" xr:uid="{1AA839FE-7FAE-4414-89EC-EE37E17E27B6}"/>
+    <hyperlink ref="H32" r:id="rId44" xr:uid="{8920AF35-BAAB-4C2A-B1BC-98F0255C4797}"/>
+    <hyperlink ref="H34" r:id="rId45" xr:uid="{C4D06269-938A-498A-88B2-93547914AA0E}"/>
+    <hyperlink ref="D20" r:id="rId46" xr:uid="{5FEB7EF6-9CFD-E646-85D6-B3F799324D32}"/>
+    <hyperlink ref="F20" r:id="rId47" xr:uid="{1FC77F03-A110-444D-AD26-331FDC033577}"/>
+    <hyperlink ref="H20" r:id="rId48" xr:uid="{9DDCC08E-E0BC-534F-8C91-2227D361EEBD}"/>
+    <hyperlink ref="D3" r:id="rId49" display="http://snomed.info/id/91723000" xr:uid="{EE85211B-E66C-7C43-BD27-E0D2E34610FA}"/>
+    <hyperlink ref="F3" r:id="rId50" xr:uid="{F8AD7288-E608-5F4B-950D-BE7EBFF84053}"/>
+    <hyperlink ref="D38" r:id="rId51" xr:uid="{B66E6909-1AA9-F942-B78E-78B90A2BD495}"/>
+    <hyperlink ref="F38" r:id="rId52" xr:uid="{69982AA4-CE83-1D47-B0FF-D97762669A47}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId46"/>
+  <legacyDrawing r:id="rId53"/>
   <tableParts count="1">
-    <tablePart r:id="rId47"/>
+    <tablePart r:id="rId54"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>